<commit_message>
ERP3 con dominio https://jpecina.duckdns.org + Excel v28
</commit_message>
<xml_diff>
--- a/public/inventario-proyectos.xlsx
+++ b/public/inventario-proyectos.xlsx
@@ -8,11 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diferencias" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos v27" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos v28" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servidor" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Proyectos v27'!$A$1:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Proyectos v28'!$A$1:$I$53</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Servidor'!$A$1:$E$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2930,7 +2930,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="32" customHeight="1">
+    <row r="53" ht="40" customHeight="1">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>— sin despliegue —</t>
@@ -2953,7 +2953,7 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Desplegado en servidor propio: http://143.47.63.169/erp3/login (verificado 200 el 2026-10-17; solo HTTP, HTTPS no responde)</t>
+          <t>Desplegado en servidor propio con dominio y HTTPS: https://jpecina.duckdns.org/erp3/login (verificado 200 el 2026-10-17).</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">

</xml_diff>